<commit_message>
added fit results and info button
</commit_message>
<xml_diff>
--- a/data/data_M2_example.xlsx
+++ b/data/data_M2_example.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://elibeamlines-my.sharepoint.com/personal/robert_boge_eli-beams_eu/Documents/Dokumenty/07 Software/Python/2026_Laser_Beam/web_apps/streamlit_M2/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="55" documentId="8_{8B452ACB-C0F7-4244-98FF-C8A66C82152D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8251B5AC-B588-490B-88B6-1F43A46027CD}"/>
+  <xr:revisionPtr revIDLastSave="58" documentId="8_{8B452ACB-C0F7-4244-98FF-C8A66C82152D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0A42067D-E5BF-4B70-92B8-661D0E0120CA}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13872" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -72,7 +72,7 @@
     <t>Y</t>
   </si>
   <si>
-    <t>not bad, not great, 👾</t>
+    <t>not bad, not great</t>
   </si>
 </sst>
 </file>
@@ -398,6 +398,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H30"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <cols>
+    <col min="1" max="1" width="11.20703125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" t="s">

</xml_diff>